<commit_message>
Optional space passcode; tester guide covers sharing and passcodes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agamya-Test-Sheet.xlsx
+++ b/docs/Agamya-Test-Sheet.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$H$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -663,7 +663,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>The policies are titled plainly (no "template"). After accepting you reach Home.</t>
+          <t>The policies are titled plainly (no "template"). After accepting you reach Home, with Start buttons and your recent sessions.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1566,22 +1566,22 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Impact</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Menu → Impact</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Open the page after a session.</t>
+          <t>As the expert, press Yes, that's how it works.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Real counts: minutes captured, questions asked, maps confirmed, stops in practice, agent checks, languages and AI cost. Missing data says "not enough data yet".</t>
+          <t>Agamya asks "Who should learn from this?": Everyone in the space, chosen groups and people, or only me.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1595,27 +1595,27 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Groups → create a group. Then KT missions → New mission.</t>
+          <t>Choose Only me. Sign in as the second account (a learner) and open Learning.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>The new group appears under Receiver groups. The step pills are small, not tall arches.</t>
+          <t>The map's title is listed under "Other Work Maps in this space" with Request access; it cannot be opened.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -1629,27 +1629,27 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>People (or Administration) → invite an email → Create invitation.</t>
+          <t>Press Request access. As the expert (or a space admin or coordinator), open the inbox and press Share with them.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Send with Gmail opens Gmail with the message written; Copy link works. Agamya sends nothing itself.</t>
+          <t>The learner is notified and the map appears under "Work Maps you can learn from".</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1663,27 +1663,27 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Open the invitation link in a private window.</t>
+          <t>As the expert, press Share on the map and choose a group.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>It names the space and says whether to create a password or use your existing one. There is no separate space password.</t>
+          <t>Only members of that group (plus the expert and admins) can open it.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1697,27 +1697,27 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>As a learner with nothing shared, open Learning → Ask a teacher to share.</t>
+          <t>As the learner, ask a question on the Learning page about the shared map.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>"Request sent". The teacher sees it in the inbox with Share selected / Decline, and you are told the outcome.</t>
+          <t>Ask answers from the Work Map, quoting the expert, instead of "nothing approved".</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1731,27 +1731,27 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Capture a skill → Delete on a skill, and confirm.</t>
+          <t>Create a second space from Spaces and open its inbox.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>It disappears from the list.</t>
+          <t>Only that space's notifications are listed; other spaces show only an unread count with Switch.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -1762,9 +1762,383 @@
       <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="4" t="inlineStr"/>
     </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Sharing and access</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Look at your name chip in a space you created.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Your role reads "owner · admin".</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Space passcode (optional)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Spaces page, as the space owner</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Set a passcode of at least 6 characters.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>"Passcode saved". Your own session stays open.</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Space passcode (optional)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Spaces page, as the space owner</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Sign in as another member of that space.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>"&lt;space&gt; is locked": they must enter the passcode once; a wrong one is refused.</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Space passcode (optional)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Spaces page, as the space owner</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Enter the right passcode.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>The space opens (policies first if they are new). Other spaces are not affected.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Space passcode (optional)</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Spaces page, as the space owner</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>As the owner, change the passcode.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Everyone else must enter the new one.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Menu → Impact</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Open the page after a session.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Real counts: minutes captured, questions asked, maps confirmed, stops in practice, agent checks, languages and AI cost. Missing data says "not enough data yet".</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Groups → create a group. Then KT missions → New mission.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>The new group appears under Receiver groups. The step pills are small, not tall arches.</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>People (or Administration) → invite an email → Create invitation.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Send with Gmail opens Gmail with the message written; Copy link works. Agamya sends nothing itself.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Open the invitation link in a private window.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>It names the space and says whether to create a password or use your existing one. There is no separate space password.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>12.4</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>As a learner with nothing shared, open Learning → Ask a teacher to share.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>"Request sent". The teacher sees it in the inbox with Share selected / Decline, and you are told the outcome.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Capture a skill → Delete on a skill, and confirm.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>It disappears from the list.</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr"/>
+      <c r="H50" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H39"/>
-  <conditionalFormatting sqref="F5:F39">
+  <autoFilter ref="A4:H50"/>
+  <conditionalFormatting sqref="F5:F50">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1776,7 +2150,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1815,7 +2189,7 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF(Tests!F5:F39,"Pass")</f>
+        <f>COUNTIF(Tests!F5:F50,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -1826,7 +2200,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF(Tests!F5:F39,"Fail")</f>
+        <f>COUNTIF(Tests!F5:F50,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -1837,7 +2211,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Tests!F5:F39,"Blocked")</f>
+        <f>COUNTIF(Tests!F5:F50,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -1848,7 +2222,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Tests!F5:F39,"Not run")</f>
+        <f>COUNTIF(Tests!F5:F50,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -1859,7 +2233,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTA(Tests!A5:A39)</f>
+        <f>COUNTA(Tests!A5:A50)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Practise with the camera, phones, and removing people
- Practice: Start with my camera (or Share my screen); Moti is told it
  watches hands, tools and materials; Switch camera on phones.
- Phones and tablets cannot share a screen from a browser: the option is
  shown as unavailable with the reason, and capture offers the camera.
- iPhone Safari: audio contexts are created inside the tap so Moti's
  voice plays; the real microphone rate is sent when 16 kHz is refused.
- Owners and admins remove people from a space (access ends at once,
  groups left, contributions kept; owner rules enforced).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agamya-Test-Sheet.xlsx
+++ b/docs/Agamya-Test-Sheet.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$H$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$H$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -721,7 +721,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Home → Start with your screen</t>
+          <t>Home → Start with your screen (on a computer)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Home → Start with your screen</t>
+          <t>Home → Start with your screen (on a computer)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Home → Start with your screen</t>
+          <t>Home → Start with your screen (on a computer)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Home → Start with your screen</t>
+          <t>Home → Start with your screen (on a computer)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Home → Start with your screen</t>
+          <t>Home → Start with your screen (on a computer)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1338,12 +1338,12 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Choose ಕನ್ನಡ (Kannada) or हिन्दी (Hindi) and share your screen.</t>
+          <t>Choose ಕನ್ನಡ (Kannada) or हिन्दी (Hindi) and press Start with my camera (on a phone) or Share my screen (on a computer).</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Moti greets you in that language.</t>
+          <t>Moti greets you in that language. On a phone, Share my screen is shown as unavailable instead of failing.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1372,12 +1372,12 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Start doing the task the wrong way, e.g. say "I'm posting this 72,000 invoice now".</t>
+          <t>During camera practice on a phone, press Switch camera.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Moti stops you ("... would stop here. Why do you think?") and can show the expert's screen moment.</t>
+          <t>The picture switches between the back and the front camera.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Say "I'm finished" (or press I'm finished).</t>
+          <t>Start doing the task the wrong way, e.g. say "I'm posting this 72,000 invoice now".</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>A summary appears: handled well, practise next, and "not a certification".</t>
+          <t>Moti stops you ("... would stop here. Why do you think?") and can show the expert's screen moment.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1425,27 +1425,27 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>AI agents that stop where the expert would stop</t>
+          <t>Practise with Moti as tutor</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Confirmed Work Map → Use this Work Map with AI agents</t>
+          <t>Confirmed Work Map → Practise this</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Type "Post invoice INV-204 for 72,000 rupees" and press Would … stop here?</t>
+          <t>Say "I'm finished" (or press I'm finished).</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>A verdict (Stop / Ask a person / Proceed / Not covered) with the expert's own words.</t>
+          <t>A summary appears: handled well, practise next, and "not a certification".</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1459,7 +1459,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1474,12 +1474,12 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Try a routine action, e.g. a small invoice from a known supplier.</t>
+          <t>Type "Post invoice INV-204 for 72,000 rupees" and press Would … stop here?</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Proceed, naming the step.</t>
+          <t>A verdict (Stop / Ask a person / Proceed / Not covered) with the expert's own words.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Open Connect an agent, name it, press Create a key.</t>
+          <t>Try a routine action, e.g. a small invoice from a known supplier.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>A key is shown once, with MCP and REST instructions.</t>
+          <t>Proceed, naming the step.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1542,12 +1542,12 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Press Revoke on that key and confirm.</t>
+          <t>Open Connect an agent, name it, press Create a key.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>It is marked revoked.</t>
+          <t>A key is shown once, with MCP and REST instructions.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -1561,27 +1561,27 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Sharing and access</t>
+          <t>AI agents that stop where the expert would stop</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>A confirmed Work Map; a second account invited to the same space</t>
+          <t>Confirmed Work Map → Use this Work Map with AI agents</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>As the expert, press Yes, that's how it works.</t>
+          <t>Press Revoke on that key and confirm.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Agamya asks "Who should learn from this?": Everyone in the space, chosen groups and people, or only me.</t>
+          <t>It is marked revoked.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Choose Only me. Sign in as the second account (a learner) and open Learning.</t>
+          <t>As the expert, press Yes, that's how it works.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>The map's title is listed under "Other Work Maps in this space" with Request access; it cannot be opened.</t>
+          <t>Agamya asks "Who should learn from this?": Everyone in the space, chosen groups and people, or only me.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -1629,7 +1629,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1644,12 +1644,12 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Press Request access. As the expert (or a space admin or coordinator), open the inbox and press Share with them.</t>
+          <t>Choose Only me. Sign in as the second account (a learner) and open Learning.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>The learner is notified and the map appears under "Work Maps you can learn from".</t>
+          <t>The map's title is listed under "Other Work Maps in this space" with Request access; it cannot be opened.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1663,7 +1663,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>As the expert, press Share on the map and choose a group.</t>
+          <t>Press Request access. As the expert (or a space admin or coordinator), open the inbox and press Share with them.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Only members of that group (plus the expert and admins) can open it.</t>
+          <t>The learner is notified and the map appears under "Work Maps you can learn from".</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>As the learner, ask a question on the Learning page about the shared map.</t>
+          <t>As the expert, press Share on the map and choose a group.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Ask answers from the Work Map, quoting the expert, instead of "nothing approved".</t>
+          <t>Only members of that group (plus the expert and admins) can open it.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1731,7 +1731,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Create a second space from Spaces and open its inbox.</t>
+          <t>As the learner, ask a question on the Learning page about the shared map.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Only that space's notifications are listed; other spaces show only an unread count with Switch.</t>
+          <t>Ask answers from the Work Map, quoting the expert, instead of "nothing approved".</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -1765,7 +1765,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -1780,12 +1780,12 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Look at your name chip in a space you created.</t>
+          <t>Create a second space from Spaces and open its inbox.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Your role reads "owner · admin".</t>
+          <t>Only that space's notifications are listed; other spaces show only an unread count with Switch.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -1799,27 +1799,27 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Space passcode (optional)</t>
+          <t>Sharing and access</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Spaces page, as the space owner</t>
+          <t>A confirmed Work Map; a second account invited to the same space</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Set a passcode of at least 6 characters.</t>
+          <t>Look at your name chip in a space you created.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>"Passcode saved". Your own session stays open.</t>
+          <t>Your role reads "owner · admin".</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -1833,7 +1833,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Sign in as another member of that space.</t>
+          <t>Set a passcode of at least 6 characters.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>"&lt;space&gt; is locked": they must enter the passcode once; a wrong one is refused.</t>
+          <t>"Passcode saved". Your own session stays open.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -1867,7 +1867,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -1882,12 +1882,12 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Enter the right passcode.</t>
+          <t>Sign in as another member of that space.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>The space opens (policies first if they are new). Other spaces are not affected.</t>
+          <t>"&lt;space&gt; is locked": they must enter the passcode once; a wrong one is refused.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -1916,12 +1916,12 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>As the owner, change the passcode.</t>
+          <t>Enter the right passcode.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Everyone else must enter the new one.</t>
+          <t>The space opens (policies first if they are new). Other spaces are not affected.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Impact</t>
+          <t>Space passcode (optional)</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Menu → Impact</t>
+          <t>Spaces page, as the space owner</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Open the page after a session.</t>
+          <t>As the owner, change the passcode.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Real counts: minutes captured, questions asked, maps confirmed, stops in practice, agent checks, languages and AI cost. Missing data says "not enough data yet".</t>
+          <t>Everyone else must enter the new one.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -1969,27 +1969,27 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Spaces, people and sharing</t>
+          <t>Impact</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Work judge for missions; Culture judge for sharing</t>
+          <t>Menu → Impact</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Groups → create a group. Then KT missions → New mission.</t>
+          <t>Open the page after a session.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>The new group appears under Receiver groups. The step pills are small, not tall arches.</t>
+          <t>Real counts: minutes captured, questions asked, maps confirmed, stops in practice, agent checks, languages and AI cost. Missing data says "not enough data yet".</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -2018,12 +2018,12 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>People (or Administration) → invite an email → Create invitation.</t>
+          <t>Groups → create a group. Then KT missions → New mission.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Send with Gmail opens Gmail with the message written; Copy link works. Agamya sends nothing itself.</t>
+          <t>The new group appears under Receiver groups. The step pills are small, not tall arches.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2037,7 +2037,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Open the invitation link in a private window.</t>
+          <t>People (or Administration) → invite an email → Create invitation.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>It names the space and says whether to create a password or use your existing one. There is no separate space password.</t>
+          <t>Send with Gmail opens Gmail with the message written; Copy link works. Agamya sends nothing itself.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -2071,7 +2071,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>As a learner with nothing shared, open Learning → Ask a teacher to share.</t>
+          <t>Open the invitation link in a private window.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>"Request sent". The teacher sees it in the inbox with Share selected / Decline, and you are told the outcome.</t>
+          <t>It names the space and says whether to create a password or use your existing one. There is no separate space password.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -2105,7 +2105,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.4</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Capture a skill → Delete on a skill, and confirm.</t>
+          <t>As a learner with nothing shared, open Learning → Ask a teacher to share.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>It disappears from the list.</t>
+          <t>"Request sent". The teacher sees it in the inbox with Share selected / Decline, and you are told the outcome.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -2136,9 +2136,77 @@
       <c r="G50" s="4" t="inlineStr"/>
       <c r="H50" s="4" t="inlineStr"/>
     </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Capture a skill → Delete on a skill, and confirm.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>It disappears from the list.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>12.6</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Spaces, people and sharing</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Work judge for missions; Culture judge for sharing</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>As an owner or admin, open People (or Administration) and press Remove from space on a member, then confirm.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>They disappear from the list and from sharing choices; their access to the space ends at once. Only the owner can remove an owner or admin.</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr"/>
+      <c r="H52" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H50"/>
-  <conditionalFormatting sqref="F5:F50">
+  <autoFilter ref="A4:H52"/>
+  <conditionalFormatting sqref="F5:F52">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2150,7 +2218,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2189,7 +2257,7 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF(Tests!F5:F50,"Pass")</f>
+        <f>COUNTIF(Tests!F5:F52,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -2200,7 +2268,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF(Tests!F5:F50,"Fail")</f>
+        <f>COUNTIF(Tests!F5:F52,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -2211,7 +2279,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Tests!F5:F50,"Blocked")</f>
+        <f>COUNTIF(Tests!F5:F52,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -2222,7 +2290,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Tests!F5:F50,"Not run")</f>
+        <f>COUNTIF(Tests!F5:F52,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -2233,7 +2301,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTA(Tests!A5:A50)</f>
+        <f>COUNTA(Tests!A5:A52)</f>
         <v/>
       </c>
     </row>

</xml_diff>